<commit_message>
math functions, shapes & other factors. tommorow trying to import specific battery types into main file
</commit_message>
<xml_diff>
--- a/CDCM Requirements.xlsx
+++ b/CDCM Requirements.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rashijainx/Documents/GitHub/lunar_habitat_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA04B718-B295-C741-81DB-AD56BEEE3030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9687B284-22C7-8F42-83BD-D4E2D39338D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{68C7D032-9CC6-2342-A3A6-13E43AA40885}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{68C7D032-9CC6-2342-A3A6-13E43AA40885}"/>
   </bookViews>
   <sheets>
     <sheet name="High Level Requirements " sheetId="1" r:id="rId1"/>
     <sheet name="Core Level Requirements" sheetId="2" r:id="rId2"/>
+    <sheet name="Exterior Structure " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -456,4 +457,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7875A8D6-EC08-4C44-A899-C7650EB2155F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>